<commit_message>
Redesign Churches page: parse new Excel data into State->District->Church Name->Pastor->Address hierarchy with Classic & Responsible UI styling
</commit_message>
<xml_diff>
--- a/churches-state and district wise/MISSIONARY DETAILS ALL FINAL.xlsx
+++ b/churches-state and district wise/MISSIONARY DETAILS ALL FINAL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akash\AppData\Local\Packages\5319275A.WhatsAppDesktop_cv1g1gvanyjgm\LocalState\sessions\43A54D5B1BC26064400CD7281476B5F5D232C2CE\transfers\2026-09\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CEFM CHURCH\churches-state and district wise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759E4219-CDB9-4696-8E45-20D258846BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4435CED5-8146-4D83-82BF-E84B432A8898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANDHRA PRADESH" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="248">
   <si>
     <t>NO</t>
   </si>
@@ -670,9 +670,6 @@
     <t>ATHINARAYANAPURAM,MELATHERU-PO,ALLAPAKKAM VALI, KURINPADI-TK KADALORE-DIST</t>
   </si>
   <si>
-    <t>STEPHAN P NAGARAJ.BATTC</t>
-  </si>
-  <si>
     <t>303,SC STREET, THALIGAIVIDUTHY,THANJUR-DIST</t>
   </si>
   <si>
@@ -724,13 +721,70 @@
     <t>Pr.VIMALRAJ</t>
   </si>
   <si>
-    <t>NADUVELI, KATHIRAMANGALAM,TANJORE-DIST</t>
-  </si>
-  <si>
-    <t>S. SIMEON JEBARAJ</t>
-  </si>
-  <si>
-    <t>MAANA RAJA KOVIL ST,THISAYANVILAI,TIRUNELVELI-DIST</t>
+    <t>CEFM Yesu Azhaikiraar Prayer House</t>
+  </si>
+  <si>
+    <t>CEFM Witness Tabernacle Church</t>
+  </si>
+  <si>
+    <t>CEFM Church</t>
+  </si>
+  <si>
+    <t>CEFM Parisuthar Devalayam</t>
+  </si>
+  <si>
+    <t>CEFM Magimai Rajaavin Sabai</t>
+  </si>
+  <si>
+    <t>CEFM Vaanathin Vaasal Jebaveedu</t>
+  </si>
+  <si>
+    <t>CEFM Devadarisana Thirusabai</t>
+  </si>
+  <si>
+    <t>NARUVELI, KATHIRAMANGALAM,TANJORE-DIST</t>
+  </si>
+  <si>
+    <t>A. SIMEON JEBARAJ</t>
+  </si>
+  <si>
+    <t>CEFM Worship Tabernacle</t>
+  </si>
+  <si>
+    <t>STEPHAN P NAGARAJ</t>
+  </si>
+  <si>
+    <t>CEFM church</t>
+  </si>
+  <si>
+    <t>MARIYADAS</t>
+  </si>
+  <si>
+    <t>KADALANGUDI,MAYILADUTHURAI,NAGAI-DIST</t>
+  </si>
+  <si>
+    <t>CEFM Karthar Jeevanullor Jebaveedu</t>
+  </si>
+  <si>
+    <t>YACOB</t>
+  </si>
+  <si>
+    <t>KAATHIRUPPu,NAGAI-DIST</t>
+  </si>
+  <si>
+    <t>DAVID</t>
+  </si>
+  <si>
+    <t>BANDIREVU,BHADRACHALAM MANDAL,KHAMMAM.</t>
+  </si>
+  <si>
+    <t>AANJANEYALU</t>
+  </si>
+  <si>
+    <t>BALAGI NAGAR</t>
+  </si>
+  <si>
+    <t>CHURCH NAME</t>
   </si>
 </sst>
 </file>
@@ -1051,14 +1105,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="35.5546875" customWidth="1"/>
     <col min="3" max="3" width="67.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1068,8 +1123,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1079,8 +1137,11 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1090,8 +1151,11 @@
       <c r="C3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1101,8 +1165,11 @@
       <c r="C4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1112,8 +1179,11 @@
       <c r="C5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1123,8 +1193,11 @@
       <c r="C6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1134,8 +1207,11 @@
       <c r="C7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1145,8 +1221,11 @@
       <c r="C8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1156,8 +1235,11 @@
       <c r="C9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1167,8 +1249,11 @@
       <c r="C10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1178,8 +1263,11 @@
       <c r="C11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1189,8 +1277,11 @@
       <c r="C12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1200,8 +1291,11 @@
       <c r="C13" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1211,8 +1305,11 @@
       <c r="C14" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1222,8 +1319,11 @@
       <c r="C15" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1233,8 +1333,11 @@
       <c r="C16" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1244,8 +1347,11 @@
       <c r="C17" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1255,8 +1361,11 @@
       <c r="C18" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1266,8 +1375,11 @@
       <c r="C19" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1277,8 +1389,11 @@
       <c r="C20" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1288,8 +1403,11 @@
       <c r="C21" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1299,8 +1417,11 @@
       <c r="C22" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1310,8 +1431,11 @@
       <c r="C23" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D23" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1321,8 +1445,11 @@
       <c r="C24" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D24" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1332,8 +1459,11 @@
       <c r="C25" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D25" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1343,8 +1473,11 @@
       <c r="C26" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D26" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1354,8 +1487,11 @@
       <c r="C27" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D27" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1365,23 +1501,41 @@
       <c r="C28" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>243</v>
+      </c>
+      <c r="C29" t="s">
+        <v>244</v>
+      </c>
+      <c r="D29" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>245</v>
+      </c>
+      <c r="C30" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1408,14 +1562,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
     <col min="3" max="3" width="80.21875" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1425,8 +1580,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1436,8 +1594,11 @@
       <c r="C2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1447,8 +1608,11 @@
       <c r="C3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1458,8 +1622,11 @@
       <c r="C4" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1469,8 +1636,11 @@
       <c r="C5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1480,8 +1650,11 @@
       <c r="C6" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1491,8 +1664,11 @@
       <c r="C7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1502,8 +1678,11 @@
       <c r="C8" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1513,8 +1692,11 @@
       <c r="C9" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1524,8 +1706,11 @@
       <c r="C10" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1535,8 +1720,11 @@
       <c r="C11" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1546,8 +1734,11 @@
       <c r="C12" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1557,8 +1748,11 @@
       <c r="C13" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1568,8 +1762,11 @@
       <c r="C14" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1579,8 +1776,11 @@
       <c r="C15" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1590,8 +1790,11 @@
       <c r="C16" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1601,8 +1804,11 @@
       <c r="C17" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1612,8 +1818,11 @@
       <c r="C18" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1623,8 +1832,11 @@
       <c r="C19" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1634,8 +1846,11 @@
       <c r="C20" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1645,8 +1860,11 @@
       <c r="C21" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1656,8 +1874,11 @@
       <c r="C22" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1667,8 +1888,11 @@
       <c r="C23" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D23" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1677,6 +1901,9 @@
       </c>
       <c r="C24" t="s">
         <v>100</v>
+      </c>
+      <c r="D24" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -1686,14 +1913,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
     <col min="3" max="3" width="74.5546875" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1703,8 +1931,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1714,8 +1945,11 @@
       <c r="C2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1725,8 +1959,11 @@
       <c r="C3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1736,8 +1973,11 @@
       <c r="C4" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1747,8 +1987,11 @@
       <c r="C5" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1758,8 +2001,11 @@
       <c r="C6" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1769,8 +2015,11 @@
       <c r="C7" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1780,8 +2029,11 @@
       <c r="C8" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1791,8 +2043,11 @@
       <c r="C9" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1802,8 +2057,11 @@
       <c r="C10" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1813,8 +2071,11 @@
       <c r="C11" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1824,8 +2085,11 @@
       <c r="C12" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1835,8 +2099,11 @@
       <c r="C13" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1846,8 +2113,11 @@
       <c r="C14" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1857,8 +2127,11 @@
       <c r="C15" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1868,8 +2141,11 @@
       <c r="C16" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1879,8 +2155,11 @@
       <c r="C17" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1890,8 +2169,11 @@
       <c r="C18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1900,6 +2182,9 @@
       </c>
       <c r="C19" t="s">
         <v>161</v>
+      </c>
+      <c r="D19" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -1909,14 +2194,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="66.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -1926,8 +2212,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1937,8 +2226,11 @@
       <c r="C2" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1948,8 +2240,11 @@
       <c r="C3" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1959,8 +2254,11 @@
       <c r="C4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1970,8 +2268,11 @@
       <c r="C5" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1981,8 +2282,11 @@
       <c r="C6" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1992,8 +2296,11 @@
       <c r="C7" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2011,14 +2318,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="43.5546875" customWidth="1"/>
     <col min="3" max="3" width="61.88671875" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2028,8 +2336,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2039,8 +2350,11 @@
       <c r="C2" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2050,8 +2364,11 @@
       <c r="C3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2061,8 +2378,11 @@
       <c r="C4" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2072,8 +2392,11 @@
       <c r="C5" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2083,8 +2406,11 @@
       <c r="C6" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2094,8 +2420,11 @@
       <c r="C7" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2105,8 +2434,11 @@
       <c r="C8" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2116,8 +2448,11 @@
       <c r="C9" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2127,8 +2462,11 @@
       <c r="C10" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2138,8 +2476,11 @@
       <c r="C11" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2149,8 +2490,11 @@
       <c r="C12" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2159,6 +2503,9 @@
       </c>
       <c r="C13" t="s">
         <v>174</v>
+      </c>
+      <c r="D13" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -2168,14 +2515,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.21875" customWidth="1"/>
     <col min="3" max="3" width="78.109375" customWidth="1"/>
+    <col min="4" max="4" width="50.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2185,8 +2533,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2196,8 +2547,11 @@
       <c r="C2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2207,8 +2561,11 @@
       <c r="C3" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2218,8 +2575,11 @@
       <c r="C4" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2229,8 +2589,11 @@
       <c r="C5" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2240,8 +2603,11 @@
       <c r="C6" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2251,8 +2617,11 @@
       <c r="C7" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2262,8 +2631,11 @@
       <c r="C8" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2273,8 +2645,11 @@
       <c r="C9" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2284,8 +2659,11 @@
       <c r="C10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2295,8 +2673,11 @@
       <c r="C11" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2306,19 +2687,25 @@
       <c r="C12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>225</v>
+      </c>
+      <c r="C13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D13" t="s">
         <v>226</v>
       </c>
-      <c r="C13" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2328,8 +2715,11 @@
       <c r="C14" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2339,8 +2729,11 @@
       <c r="C15" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2350,8 +2743,11 @@
       <c r="C16" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2361,19 +2757,25 @@
       <c r="C17" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C18" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>224</v>
+      </c>
+      <c r="D18" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2383,8 +2785,11 @@
       <c r="C19" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2394,119 +2799,158 @@
       <c r="C20" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>236</v>
+      </c>
+      <c r="C21" t="s">
         <v>209</v>
       </c>
-      <c r="C21" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>210</v>
+      </c>
+      <c r="C22" t="s">
         <v>211</v>
       </c>
-      <c r="C22" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>238</v>
+      </c>
+      <c r="C23" t="s">
+        <v>239</v>
+      </c>
+      <c r="D23" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
-        <v>228</v>
-      </c>
-      <c r="C24" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C25" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+      <c r="D25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>213</v>
+      </c>
+      <c r="C27" t="s">
         <v>214</v>
       </c>
-      <c r="C27" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D27" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>215</v>
+      </c>
+      <c r="C28" t="s">
         <v>216</v>
       </c>
-      <c r="C28" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>217</v>
+      </c>
+      <c r="C29" t="s">
         <v>218</v>
       </c>
-      <c r="C29" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>241</v>
+      </c>
+      <c r="C30" t="s">
+        <v>242</v>
+      </c>
+      <c r="D30" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C31" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+        <v>223</v>
+      </c>
+      <c r="D31" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>220</v>
+      </c>
+      <c r="C32" t="s">
         <v>221</v>
       </c>
-      <c r="C32" t="s">
-        <v>222</v>
+      <c r="D32" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: navbar layout, favicon, live stream, footer Reach Us, prayer email, Google Maps, Telangana photos
</commit_message>
<xml_diff>
--- a/churches-state and district wise/MISSIONARY DETAILS ALL FINAL.xlsx
+++ b/churches-state and district wise/MISSIONARY DETAILS ALL FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CEFM CHURCH\churches-state and district wise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4435CED5-8146-4D83-82BF-E84B432A8898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169C137E-1C05-4695-B2D7-23788E10914E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANDHRA PRADESH" sheetId="1" r:id="rId1"/>
@@ -577,9 +577,6 @@
     <t>P. SATHROCK</t>
   </si>
   <si>
-    <t>ERUMOOLI MELA WELI, THIRUVADIMARUZHUR-T.K, KOZHOLAMPALLAM, TANJORE.</t>
-  </si>
-  <si>
     <t>S. PETER</t>
   </si>
   <si>
@@ -589,9 +586,6 @@
     <t>B. BASKAR</t>
   </si>
   <si>
-    <t>KILINSEL STREET,NATARAJAPURAM,CHIDAMBARAM,DIST-CUDALORE.</t>
-  </si>
-  <si>
     <t>K. PHILIP VIJENDRAN</t>
   </si>
   <si>
@@ -601,15 +595,9 @@
     <t>S. SARAL</t>
   </si>
   <si>
-    <t>MELATHERU,KONULAM PALLAM,ANAKKARAI,TANJAVORE-DIST</t>
-  </si>
-  <si>
     <t>S. JOHNWESLEY</t>
   </si>
   <si>
-    <t xml:space="preserve">55A,BITTHAR,GANDHINAGAR,VELLER,SATTHUVA NAGAR,VELLER-DISTM. </t>
-  </si>
-  <si>
     <t>HOSPITAL STREET,PALANGUR,TIRUKOILLUR,DIST-VILLUPURAM</t>
   </si>
   <si>
@@ -637,9 +625,6 @@
     <t>R. DANIEL</t>
   </si>
   <si>
-    <t>PUTHU THERU,KADDUMANNARKOVIL,VEERANANTHAPURAM, KADALLOR-DIST</t>
-  </si>
-  <si>
     <t>P. SAMUELMANI</t>
   </si>
   <si>
@@ -655,33 +640,15 @@
     <t>R. SEKAR(DANIEL)</t>
   </si>
   <si>
-    <t>MAIN ROAD, KOMAL-PO,KUTTALAM.</t>
-  </si>
-  <si>
     <t>K.K. DEVASELVAM</t>
   </si>
   <si>
-    <t>1/76E,MANTHAKARI,KUMARAMANGALAM,CHIDAMBARAM,CUDALORE-DIST.</t>
-  </si>
-  <si>
     <t>T. SATHRAK</t>
   </si>
   <si>
-    <t>ATHINARAYANAPURAM,MELATHERU-PO,ALLAPAKKAM VALI, KURINPADI-TK KADALORE-DIST</t>
-  </si>
-  <si>
-    <t>303,SC STREET, THALIGAIVIDUTHY,THANJUR-DIST</t>
-  </si>
-  <si>
     <t>M. ARULDASS</t>
   </si>
   <si>
-    <t>BETHEL ST,SIKKALNAYAKKAN PATTAI,THANJAVUR-DIST</t>
-  </si>
-  <si>
-    <t>5/5, RAILWAY STATION, POONGULATHUVILLAI,KANYAKUMAI-DIST</t>
-  </si>
-  <si>
     <t>K. SANTHOSAM</t>
   </si>
   <si>
@@ -706,18 +673,9 @@
     <t>P. GIDEON MUNIYANDI</t>
   </si>
   <si>
-    <t>1/14,MATHA KAVELI ST,AAGARAM,ARANI,VENAMAGAIM,T.V.MALI DIST.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rev.S. HUBERT SUBIN RAJ </t>
   </si>
   <si>
-    <t>3/6,PALLIKOODATHERU,ECHAMPOONDI,KATTUMANNARKOVIL,CADALLORE-DIST</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> KARTUMANNARKOVIL ,VEERANATHAM,CUDALORE-DIST</t>
-  </si>
-  <si>
     <t>Pr.VIMALRAJ</t>
   </si>
   <si>
@@ -785,6 +743,48 @@
   </si>
   <si>
     <t>CHURCH NAME</t>
+  </si>
+  <si>
+    <t>ERUMOOLI MELA WELI, THIRUVADIMARUZHUR-T.K, KOZHOLAMPALLAM, TANJORE-DIST</t>
+  </si>
+  <si>
+    <t>KILINSEL STREET,NATARAJAPURAM,CHIDAMBARAM,DIST-CUDDUALORE</t>
+  </si>
+  <si>
+    <t>MELATHERU,KONULAM PALLAM,ANAKKARAI,TANJORE-DIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55A,BITTHAR,GANDHINAGAR,VELLER,SATTHUVA NAGAR,VELLORE-DIST. </t>
+  </si>
+  <si>
+    <t>PUTHU THERU,KADDUMANNARKOVIL,VEERANANTHAPURAM, CUDDUALORE-DIST</t>
+  </si>
+  <si>
+    <t>MAIN ROAD, KOMAL-PO,KUTTALAM,MAYILADUTHURAI-DIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KARTUMANNARKOVIL ,VEERANATHAM,CUDDUALORE-DIST</t>
+  </si>
+  <si>
+    <t>1/76E,MANTHAKARI,KUMARAMANGALAM,CHIDAMBARAM,CUDDUALORE-DIST.</t>
+  </si>
+  <si>
+    <t>ATHINARAYANAPURAM,MELATHERU-PO,ALLAPAKKAM VALI, KURINPADI-TK CUDDUALORE-DIST</t>
+  </si>
+  <si>
+    <t>303,SC STREET, THALIGAIVIDUTHY,TANJORE-DIST</t>
+  </si>
+  <si>
+    <t>BETHEL ST,SIKKALNAYAKKAN PATTAI,TANJORE-DIST</t>
+  </si>
+  <si>
+    <t>5/5, RAILWAY STATION, POONGULATHUVILLAI,KANYAKUMARI-DIST</t>
+  </si>
+  <si>
+    <t>3/6,PALLIKOODATHERU,ECHAMPOONDI,KATTUMANNARKOVIL,CUDDUALORE-DIST</t>
+  </si>
+  <si>
+    <t>1/14,MATHA KAVELI ST,AAGARAM,ARANI,VENAMAGAIM,TIRUVANNAMALAI-DIST.</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +1124,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1138,7 +1138,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1152,7 +1152,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1166,7 +1166,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1180,7 +1180,7 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1194,7 +1194,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1208,7 +1208,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1222,7 +1222,7 @@
         <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1236,7 +1236,7 @@
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1250,7 +1250,7 @@
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1264,7 +1264,7 @@
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1278,7 +1278,7 @@
         <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1292,7 +1292,7 @@
         <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1306,7 +1306,7 @@
         <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1320,7 +1320,7 @@
         <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1334,7 +1334,7 @@
         <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1348,7 +1348,7 @@
         <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1362,7 +1362,7 @@
         <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1376,7 +1376,7 @@
         <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1390,7 +1390,7 @@
         <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1404,7 +1404,7 @@
         <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1418,7 +1418,7 @@
         <v>44</v>
       </c>
       <c r="D22" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1432,7 +1432,7 @@
         <v>44</v>
       </c>
       <c r="D23" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1446,7 +1446,7 @@
         <v>47</v>
       </c>
       <c r="D24" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1460,7 +1460,7 @@
         <v>49</v>
       </c>
       <c r="D25" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1474,7 +1474,7 @@
         <v>51</v>
       </c>
       <c r="D26" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1488,7 +1488,7 @@
         <v>53</v>
       </c>
       <c r="D27" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1502,7 +1502,7 @@
         <v>55</v>
       </c>
       <c r="D28" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1510,13 +1510,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="C29" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="D29" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1524,10 +1524,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="C30" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1581,7 +1581,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1595,7 +1595,7 @@
         <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1609,7 +1609,7 @@
         <v>57</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1623,7 +1623,7 @@
         <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1637,7 +1637,7 @@
         <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1651,7 +1651,7 @@
         <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1665,7 +1665,7 @@
         <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1679,7 +1679,7 @@
         <v>68</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1693,7 +1693,7 @@
         <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1707,7 +1707,7 @@
         <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1721,7 +1721,7 @@
         <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1735,7 +1735,7 @@
         <v>76</v>
       </c>
       <c r="D12" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1749,7 +1749,7 @@
         <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1763,7 +1763,7 @@
         <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1777,7 +1777,7 @@
         <v>82</v>
       </c>
       <c r="D15" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1791,7 +1791,7 @@
         <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1805,7 +1805,7 @@
         <v>86</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1819,7 +1819,7 @@
         <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1833,7 +1833,7 @@
         <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1847,7 +1847,7 @@
         <v>92</v>
       </c>
       <c r="D20" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1861,7 +1861,7 @@
         <v>94</v>
       </c>
       <c r="D21" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1875,7 +1875,7 @@
         <v>96</v>
       </c>
       <c r="D22" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1889,7 +1889,7 @@
         <v>98</v>
       </c>
       <c r="D23" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1903,7 +1903,7 @@
         <v>100</v>
       </c>
       <c r="D24" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -1932,7 +1932,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1946,7 +1946,7 @@
         <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1960,7 +1960,7 @@
         <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1974,7 +1974,7 @@
         <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1988,7 +1988,7 @@
         <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2002,7 +2002,7 @@
         <v>110</v>
       </c>
       <c r="D6" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -2016,7 +2016,7 @@
         <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -2030,7 +2030,7 @@
         <v>114</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -2044,7 +2044,7 @@
         <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -2058,7 +2058,7 @@
         <v>118</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -2072,7 +2072,7 @@
         <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2086,7 +2086,7 @@
         <v>122</v>
       </c>
       <c r="D12" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2100,7 +2100,7 @@
         <v>124</v>
       </c>
       <c r="D13" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -2114,7 +2114,7 @@
         <v>126</v>
       </c>
       <c r="D14" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -2128,7 +2128,7 @@
         <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -2142,7 +2142,7 @@
         <v>130</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -2156,7 +2156,7 @@
         <v>132</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -2170,7 +2170,7 @@
         <v>134</v>
       </c>
       <c r="D18" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -2184,7 +2184,7 @@
         <v>161</v>
       </c>
       <c r="D19" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -2213,7 +2213,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2227,7 +2227,7 @@
         <v>137</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2241,7 +2241,7 @@
         <v>139</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2255,7 +2255,7 @@
         <v>141</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2269,7 +2269,7 @@
         <v>143</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2283,7 +2283,7 @@
         <v>145</v>
       </c>
       <c r="D6" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -2297,7 +2297,7 @@
         <v>147</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -2337,7 +2337,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2351,7 +2351,7 @@
         <v>151</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2365,7 +2365,7 @@
         <v>153</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2379,7 +2379,7 @@
         <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2393,7 +2393,7 @@
         <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2407,7 +2407,7 @@
         <v>159</v>
       </c>
       <c r="D6" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -2421,7 +2421,7 @@
         <v>163</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -2435,7 +2435,7 @@
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -2449,7 +2449,7 @@
         <v>167</v>
       </c>
       <c r="D9" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -2463,7 +2463,7 @@
         <v>169</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -2477,7 +2477,7 @@
         <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2491,7 +2491,7 @@
         <v>172</v>
       </c>
       <c r="D12" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2505,7 +2505,7 @@
         <v>174</v>
       </c>
       <c r="D13" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -2534,7 +2534,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2548,7 +2548,7 @@
         <v>176</v>
       </c>
       <c r="D2" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2559,10 +2559,10 @@
         <v>177</v>
       </c>
       <c r="C3" t="s">
-        <v>178</v>
+        <v>234</v>
       </c>
       <c r="D3" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2570,13 +2570,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" t="s">
         <v>179</v>
       </c>
-      <c r="C4" t="s">
-        <v>180</v>
-      </c>
       <c r="D4" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2584,13 +2584,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C5" t="s">
-        <v>182</v>
+        <v>235</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2598,13 +2598,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D6" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -2612,13 +2612,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>186</v>
+        <v>236</v>
       </c>
       <c r="D7" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -2626,13 +2626,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>237</v>
       </c>
       <c r="D8" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -2640,13 +2640,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D9" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -2654,13 +2654,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D10" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -2668,13 +2668,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C11" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D11" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2682,13 +2682,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C12" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D12" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2696,13 +2696,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="C13" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="D13" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -2710,13 +2710,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C14" t="s">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="D14" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -2724,13 +2724,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C15" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D15" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -2738,13 +2738,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C16" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D16" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -2752,13 +2752,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C17" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="D17" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -2766,13 +2766,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="C18" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="D18" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -2780,13 +2780,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C19" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="D19" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -2794,13 +2794,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C20" t="s">
-        <v>208</v>
+        <v>242</v>
       </c>
       <c r="D20" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -2808,13 +2808,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="C21" t="s">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="D21" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -2822,13 +2822,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="C22" t="s">
-        <v>211</v>
+        <v>244</v>
       </c>
       <c r="D22" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -2836,13 +2836,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="C23" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="D23" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -2855,13 +2855,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C25" t="s">
-        <v>212</v>
+        <v>245</v>
       </c>
       <c r="D25" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -2874,13 +2874,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="C27" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="D27" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -2888,13 +2888,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="C28" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="D28" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -2902,13 +2902,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="C29" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="D29" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -2916,13 +2916,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="C30" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="D30" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -2930,13 +2930,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="C31" t="s">
+        <v>246</v>
+      </c>
+      <c r="D31" t="s">
         <v>223</v>
-      </c>
-      <c r="D31" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -2944,13 +2944,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C32" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="D32" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>